<commit_message>
Updated the code in invoke code activity.
</commit_message>
<xml_diff>
--- a/AP.InvoicePerformer/Data/Exports/invoice-3-3_1-2.xlsx
+++ b/AP.InvoicePerformer/Data/Exports/invoice-3-3_1-2.xlsx
@@ -28,6 +28,30 @@
     <x:t>Billing Name</x:t>
   </x:si>
   <x:si>
+    <x:t>Date</x:t>
+  </x:si>
+  <x:si>
+    <x:t>DueDate</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Invoice Number</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Shipping Charges</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Tax Amount</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Total</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Items</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Subtotal Amount</x:t>
+  </x:si>
+  <x:si>
     <x:t>Billing Address</x:t>
   </x:si>
   <x:si>
@@ -43,42 +67,18 @@
     <x:t>Vendor VAT Number</x:t>
   </x:si>
   <x:si>
-    <x:t>Date</x:t>
-  </x:si>
-  <x:si>
-    <x:t>DueDate</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Invoice Number</x:t>
-  </x:si>
-  <x:si>
     <x:t>PO Number</x:t>
   </x:si>
   <x:si>
     <x:t>Payment Terms</x:t>
   </x:si>
   <x:si>
-    <x:t>Shipping Charges</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Tax Amount</x:t>
-  </x:si>
-  <x:si>
     <x:t>Net Amount</x:t>
   </x:si>
   <x:si>
-    <x:t>Total</x:t>
-  </x:si>
-  <x:si>
     <x:t>Discount</x:t>
   </x:si>
   <x:si>
-    <x:t>Items</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Subtotal Amount</x:t>
-  </x:si>
-  <x:si>
     <x:t>Neid</x:t>
   </x:si>
   <x:si>
@@ -88,31 +88,34 @@
     <x:t>Zuuf AG</x:t>
   </x:si>
   <x:si>
+    <x:t>2021-12-22</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2022-01-22</x:t>
+  </x:si>
+  <x:si>
+    <x:t>4405</x:t>
+  </x:si>
+  <x:si>
+    <x:t>25000</x:t>
+  </x:si>
+  <x:si>
+    <x:t>74850</x:t>
+  </x:si>
+  <x:si>
+    <x:t>848350</x:t>
+  </x:si>
+  <x:si>
+    <x:t>table</x:t>
+  </x:si>
+  <x:si>
+    <x:t>748500</x:t>
+  </x:si>
+  <x:si>
     <x:t>Domsdorfer Kirchweg 14 Forst, BRB, 03149</x:t>
   </x:si>
   <x:si>
     <x:t>as recipient Domsdorfer Kirchweg 14 03149</x:t>
-  </x:si>
-  <x:si>
-    <x:t>2021-12-22</x:t>
-  </x:si>
-  <x:si>
-    <x:t>2022-01-22</x:t>
-  </x:si>
-  <x:si>
-    <x:t>4405</x:t>
-  </x:si>
-  <x:si>
-    <x:t>25000</x:t>
-  </x:si>
-  <x:si>
-    <x:t>74850</x:t>
-  </x:si>
-  <x:si>
-    <x:t>848350</x:t>
-  </x:si>
-  <x:si>
-    <x:t>table</x:t>
   </x:si>
   <x:si>
     <x:t>Key,Value
@@ -123,18 +126,7 @@
 "Zip Postal Code","83022"</x:t>
   </x:si>
   <x:si>
-    <x:t>Key,Value
-"Address Line 1","Domsdorfer Kirchweg 14 BRB"
-"City","Forst"
-"Zip Postal Code","03149"</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Key,Value
-"Address Line 1","as recipient Domsdorfer 14"
-"City","Kirchweg"
-"Country","Germany"
-"State / County / Province","Schleswig-Holstein"
-"Zip Postal Code","03149"</x:t>
+    <x:t>748500.00</x:t>
   </x:si>
   <x:si>
     <x:t>Line Number</x:t>
@@ -816,29 +808,35 @@
       <x:c r="D2" s="0" t="s">
         <x:v>23</x:v>
       </x:c>
+      <x:c r="E2" s="0" t="s">
+        <x:v>24</x:v>
+      </x:c>
       <x:c r="F2" s="0" t="s">
-        <x:v>24</x:v>
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="G2" s="0" t="s">
+        <x:v>26</x:v>
+      </x:c>
+      <x:c r="H2" s="0" t="s">
+        <x:v>27</x:v>
       </x:c>
       <x:c r="I2" s="0" t="s">
-        <x:v>25</x:v>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="J2" s="0" t="s">
-        <x:v>26</x:v>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="K2" s="0" t="s">
-        <x:v>27</x:v>
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="L2" s="0" t="s">
+        <x:v>31</x:v>
       </x:c>
       <x:c r="N2" s="0" t="s">
-        <x:v>28</x:v>
-      </x:c>
-      <x:c r="O2" s="0" t="s">
-        <x:v>29</x:v>
-      </x:c>
-      <x:c r="Q2" s="0" t="s">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="S2" s="0" t="s">
         <x:v>30</x:v>
-      </x:c>
-      <x:c r="S2" s="0" t="s">
-        <x:v>31</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -925,37 +923,43 @@
         <x:v>20</x:v>
       </x:c>
       <x:c r="B2" s="1" t="s">
-        <x:v>32</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="C2" s="0" t="s">
         <x:v>22</x:v>
       </x:c>
       <x:c r="D2" s="1" t="s">
-        <x:v>33</x:v>
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="E2" s="0" t="s">
+        <x:v>24</x:v>
       </x:c>
       <x:c r="F2" s="1" t="s">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="G2" s="0" t="s">
+        <x:v>26</x:v>
+      </x:c>
+      <x:c r="H2" s="0" t="s">
+        <x:v>27</x:v>
+      </x:c>
+      <x:c r="I2" s="0" t="s">
+        <x:v>28</x:v>
+      </x:c>
+      <x:c r="J2" s="0" t="s">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="K2" s="0" t="s">
         <x:v>34</x:v>
       </x:c>
-      <x:c r="I2" s="0" t="s">
-        <x:v>25</x:v>
-      </x:c>
-      <x:c r="J2" s="0" t="s">
-        <x:v>26</x:v>
-      </x:c>
-      <x:c r="K2" s="0" t="s">
-        <x:v>27</x:v>
+      <x:c r="L2" s="0" t="s">
+        <x:v>31</x:v>
       </x:c>
       <x:c r="N2" s="0" t="s">
-        <x:v>28</x:v>
-      </x:c>
-      <x:c r="O2" s="0" t="s">
-        <x:v>29</x:v>
-      </x:c>
-      <x:c r="Q2" s="0" t="s">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="S2" s="0" t="s">
         <x:v>30</x:v>
-      </x:c>
-      <x:c r="S2" s="0" t="s">
-        <x:v>31</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
Updated performer as gpt solution
</commit_message>
<xml_diff>
--- a/AP.InvoicePerformer/Data/Exports/invoice-3-3_1-2.xlsx
+++ b/AP.InvoicePerformer/Data/Exports/invoice-3-3_1-2.xlsx
@@ -150,49 +150,52 @@
     <x:t>Part Number</x:t>
   </x:si>
   <x:si>
+    <x:t>38700</x:t>
+  </x:si>
+  <x:si>
     <x:t>Mercury/Villager</x:t>
   </x:si>
   <x:si>
     <x:t>203-64-6102</x:t>
   </x:si>
   <x:si>
-    <x:t>38700</x:t>
-  </x:si>
-  <x:si>
     <x:t>Country of origin: Italy Color: Silver</x:t>
   </x:si>
   <x:si>
+    <x:t>35700</x:t>
+  </x:si>
+  <x:si>
     <x:t>Ford/Econoline E350</x:t>
   </x:si>
   <x:si>
     <x:t>414-85-4593</x:t>
   </x:si>
   <x:si>
-    <x:t>35700</x:t>
-  </x:si>
-  <x:si>
     <x:t>Country of origin: Germany Color: Red</x:t>
   </x:si>
   <x:si>
+    <x:t>48900</x:t>
+  </x:si>
+  <x:si>
     <x:t>Mercury/Cougar</x:t>
   </x:si>
   <x:si>
     <x:t>110-90-0753</x:t>
   </x:si>
   <x:si>
-    <x:t>48900</x:t>
-  </x:si>
-  <x:si>
     <x:t>Country of origin: Spain Color: Red</x:t>
   </x:si>
   <x:si>
+    <x:t>10900</x:t>
+  </x:si>
+  <x:si>
     <x:t>Mercedes-Benz/SL-Class</x:t>
   </x:si>
   <x:si>
     <x:t>245-29-2051</x:t>
   </x:si>
   <x:si>
-    <x:t>10900</x:t>
+    <x:t>46600</x:t>
   </x:si>
   <x:si>
     <x:t>Acura/RL</x:t>
@@ -201,34 +204,169 @@
     <x:t>374-97-8799</x:t>
   </x:si>
   <x:si>
-    <x:t>46600</x:t>
-  </x:si>
-  <x:si>
     <x:t>Country of origin: Portugal Color: Black</x:t>
   </x:si>
   <x:si>
+    <x:t>Country of origin: Spain</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Color: Blue</x:t>
+  </x:si>
+  <x:si>
+    <x:t>13500</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Jaguar/XK Series</x:t>
+  </x:si>
+  <x:si>
+    <x:t>790-94-2252</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Country of origin: Portugal</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Color: Silver</x:t>
+  </x:si>
+  <x:si>
+    <x:t>22300</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Kia/Sorento</x:t>
+  </x:si>
+  <x:si>
+    <x:t>618-41-6005</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Country of origin: Italy</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Color: Red</x:t>
+  </x:si>
+  <x:si>
+    <x:t>30900</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Ford/Bronco</x:t>
+  </x:si>
+  <x:si>
+    <x:t>877-84-8130</x:t>
+  </x:si>
+  <x:si>
+    <x:t>19000</x:t>
+  </x:si>
+  <x:si>
+    <x:t>GMC/Sierra 2500</x:t>
+  </x:si>
+  <x:si>
+    <x:t>443-68-0379</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Country of origin: Germany</x:t>
+  </x:si>
+  <x:si>
+    <x:t>30400</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Buick/Regal</x:t>
+  </x:si>
+  <x:si>
+    <x:t>667-55-8014</x:t>
+  </x:si>
+  <x:si>
+    <x:t>41400</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Volkswagen/R32</x:t>
+  </x:si>
+  <x:si>
+    <x:t>237-68-4885</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Country of origin: France</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Color: Black</x:t>
+  </x:si>
+  <x:si>
+    <x:t>21000</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Mercury/Topaz</x:t>
+  </x:si>
+  <x:si>
+    <x:t>327-67-0723</x:t>
+  </x:si>
+  <x:si>
+    <x:t>45700</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Mitsubishi/Mirage</x:t>
+  </x:si>
+  <x:si>
+    <x:t>564-51-0430</x:t>
+  </x:si>
+  <x:si>
+    <x:t>19100</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Dodge/Ram Van 3500</x:t>
+  </x:si>
+  <x:si>
+    <x:t>546-12-5620</x:t>
+  </x:si>
+  <x:si>
+    <x:t>30800</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Audi/A6</x:t>
+  </x:si>
+  <x:si>
+    <x:t>638-13-7553</x:t>
+  </x:si>
+  <x:si>
+    <x:t>22900</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Mitsubishi/Eclipse</x:t>
+  </x:si>
+  <x:si>
+    <x:t>771-81-4708</x:t>
+  </x:si>
+  <x:si>
+    <x:t>27500</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Hummer/H1</x:t>
+  </x:si>
+  <x:si>
+    <x:t>694-41-6257</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Country of origin: Germany Color: Silver</x:t>
+  </x:si>
+  <x:si>
+    <x:t>14300</x:t>
+  </x:si>
+  <x:si>
     <x:t>Oldsmobile/Custom Cruiser</x:t>
   </x:si>
   <x:si>
     <x:t>140-01-0079</x:t>
   </x:si>
   <x:si>
-    <x:t>14300</x:t>
-  </x:si>
-  <x:si>
     <x:t>Country of origin: France Color: Black</x:t>
   </x:si>
   <x:si>
+    <x:t>36000</x:t>
+  </x:si>
+  <x:si>
     <x:t>Buick/Skylark</x:t>
   </x:si>
   <x:si>
     <x:t>462-04-7728</x:t>
   </x:si>
   <x:si>
-    <x:t>36000</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Country of origin: Germany Color: Silver</x:t>
+    <x:t>28100</x:t>
   </x:si>
   <x:si>
     <x:t>Mercury/Grand Marquis</x:t>
@@ -237,31 +375,31 @@
     <x:t>870-26-8753</x:t>
   </x:si>
   <x:si>
-    <x:t>28100</x:t>
-  </x:si>
-  <x:si>
     <x:t>Country of origin: Germany Color: Blue</x:t>
   </x:si>
   <x:si>
+    <x:t>49900</x:t>
+  </x:si>
+  <x:si>
     <x:t>BMW/M5</x:t>
   </x:si>
   <x:si>
     <x:t>746-66-0334</x:t>
   </x:si>
   <x:si>
-    <x:t>49900</x:t>
-  </x:si>
-  <x:si>
     <x:t>Country of origin: Italy Color: Red</x:t>
   </x:si>
   <x:si>
+    <x:t>22600</x:t>
+  </x:si>
+  <x:si>
     <x:t>Aston Martin/V8 Vantage</x:t>
   </x:si>
   <x:si>
     <x:t>815-12-9380</x:t>
   </x:si>
   <x:si>
-    <x:t>22600</x:t>
+    <x:t>33600</x:t>
   </x:si>
   <x:si>
     <x:t>Nissan/Frontier</x:t>
@@ -270,112 +408,25 @@
     <x:t>146-53-6874</x:t>
   </x:si>
   <x:si>
-    <x:t>33600</x:t>
-  </x:si>
-  <x:si>
     <x:t>Country of origin: France Color: Red</x:t>
   </x:si>
   <x:si>
+    <x:t>18500</x:t>
+  </x:si>
+  <x:si>
     <x:t>Mitsubishi/Endeavor</x:t>
   </x:si>
   <x:si>
     <x:t>707-42-6202</x:t>
   </x:si>
   <x:si>
-    <x:t>18500</x:t>
+    <x:t>40200</x:t>
   </x:si>
   <x:si>
     <x:t>Mazda/B-Series Plus</x:t>
   </x:si>
   <x:si>
     <x:t>348-38-7014</x:t>
-  </x:si>
-  <x:si>
-    <x:t>40200</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Color: Red</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Volkswagen/R32</x:t>
-  </x:si>
-  <x:si>
-    <x:t>237-68-4885</x:t>
-  </x:si>
-  <x:si>
-    <x:t>41400</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Country of origin: France</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Color: Black</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Mercury/Topaz</x:t>
-  </x:si>
-  <x:si>
-    <x:t>327-67-0723</x:t>
-  </x:si>
-  <x:si>
-    <x:t>21000</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Country of origin: Portugal</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Color: Silver</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Mitsubishi/Mirage</x:t>
-  </x:si>
-  <x:si>
-    <x:t>564-51-0430</x:t>
-  </x:si>
-  <x:si>
-    <x:t>45700</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Country of origin: Germany</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Dodge/Ram Van 3500</x:t>
-  </x:si>
-  <x:si>
-    <x:t>546-12-5620</x:t>
-  </x:si>
-  <x:si>
-    <x:t>19100</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Audi/A6</x:t>
-  </x:si>
-  <x:si>
-    <x:t>638-13-7553</x:t>
-  </x:si>
-  <x:si>
-    <x:t>30800</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Mitsubishi/Eclipse</x:t>
-  </x:si>
-  <x:si>
-    <x:t>771-81-4708</x:t>
-  </x:si>
-  <x:si>
-    <x:t>22900</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Country of origin: Spain</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Hummer/H1</x:t>
-  </x:si>
-  <x:si>
-    <x:t>694-41-6257</x:t>
-  </x:si>
-  <x:si>
-    <x:t>27500</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -835,9 +886,6 @@
       <x:c r="N2" s="0" t="s">
         <x:v>32</x:v>
       </x:c>
-      <x:c r="S2" s="0" t="s">
-        <x:v>30</x:v>
-      </x:c>
     </x:row>
   </x:sheetData>
   <x:printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>
@@ -958,9 +1006,6 @@
       <x:c r="N2" s="0" t="s">
         <x:v>32</x:v>
       </x:c>
-      <x:c r="S2" s="0" t="s">
-        <x:v>30</x:v>
-      </x:c>
     </x:row>
   </x:sheetData>
   <x:printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>
@@ -1003,13 +1048,13 @@
       </x:c>
     </x:row>
     <x:row r="2" spans="1:7">
+      <x:c r="A2" s="0" t="s">
+        <x:v>42</x:v>
+      </x:c>
       <x:c r="B2" s="0" t="s">
-        <x:v>42</x:v>
+        <x:v>43</x:v>
       </x:c>
       <x:c r="C2" s="0" t="s">
-        <x:v>43</x:v>
-      </x:c>
-      <x:c r="E2" s="0" t="s">
         <x:v>44</x:v>
       </x:c>
     </x:row>
@@ -1019,13 +1064,13 @@
       </x:c>
     </x:row>
     <x:row r="4" spans="1:7">
+      <x:c r="A4" s="0" t="s">
+        <x:v>46</x:v>
+      </x:c>
       <x:c r="B4" s="0" t="s">
-        <x:v>46</x:v>
+        <x:v>47</x:v>
       </x:c>
       <x:c r="C4" s="0" t="s">
-        <x:v>47</x:v>
-      </x:c>
-      <x:c r="E4" s="0" t="s">
         <x:v>48</x:v>
       </x:c>
     </x:row>
@@ -1035,13 +1080,13 @@
       </x:c>
     </x:row>
     <x:row r="6" spans="1:7">
+      <x:c r="A6" s="0" t="s">
+        <x:v>50</x:v>
+      </x:c>
       <x:c r="B6" s="0" t="s">
-        <x:v>50</x:v>
+        <x:v>51</x:v>
       </x:c>
       <x:c r="C6" s="0" t="s">
-        <x:v>51</x:v>
-      </x:c>
-      <x:c r="E6" s="0" t="s">
         <x:v>52</x:v>
       </x:c>
     </x:row>
@@ -1051,13 +1096,13 @@
       </x:c>
     </x:row>
     <x:row r="8" spans="1:7">
+      <x:c r="A8" s="0" t="s">
+        <x:v>54</x:v>
+      </x:c>
       <x:c r="B8" s="0" t="s">
-        <x:v>54</x:v>
+        <x:v>55</x:v>
       </x:c>
       <x:c r="C8" s="0" t="s">
-        <x:v>55</x:v>
-      </x:c>
-      <x:c r="E8" s="0" t="s">
         <x:v>56</x:v>
       </x:c>
     </x:row>
@@ -1067,13 +1112,13 @@
       </x:c>
     </x:row>
     <x:row r="10" spans="1:7">
+      <x:c r="A10" s="0" t="s">
+        <x:v>57</x:v>
+      </x:c>
       <x:c r="B10" s="0" t="s">
-        <x:v>57</x:v>
+        <x:v>58</x:v>
       </x:c>
       <x:c r="C10" s="0" t="s">
-        <x:v>58</x:v>
-      </x:c>
-      <x:c r="E10" s="0" t="s">
         <x:v>59</x:v>
       </x:c>
     </x:row>
@@ -1086,409 +1131,391 @@
       <x:c r="B12" s="0" t="s">
         <x:v>61</x:v>
       </x:c>
-      <x:c r="C12" s="0" t="s">
-        <x:v>62</x:v>
-      </x:c>
-      <x:c r="E12" s="0" t="s">
-        <x:v>63</x:v>
-      </x:c>
     </x:row>
     <x:row r="13" spans="1:7">
       <x:c r="B13" s="0" t="s">
+        <x:v>62</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" spans="1:7">
+      <x:c r="A14" s="0" t="s">
+        <x:v>63</x:v>
+      </x:c>
+      <x:c r="B14" s="0" t="s">
         <x:v>64</x:v>
       </x:c>
-    </x:row>
-    <x:row r="14" spans="1:7">
-      <x:c r="B14" s="0" t="s">
+      <x:c r="C14" s="0" t="s">
         <x:v>65</x:v>
-      </x:c>
-      <x:c r="C14" s="0" t="s">
-        <x:v>66</x:v>
-      </x:c>
-      <x:c r="E14" s="0" t="s">
-        <x:v>67</x:v>
       </x:c>
     </x:row>
     <x:row r="15" spans="1:7">
       <x:c r="B15" s="0" t="s">
-        <x:v>68</x:v>
+        <x:v>66</x:v>
       </x:c>
     </x:row>
     <x:row r="16" spans="1:7">
       <x:c r="B16" s="0" t="s">
+        <x:v>67</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" spans="1:7">
+      <x:c r="A17" s="0" t="s">
+        <x:v>68</x:v>
+      </x:c>
+      <x:c r="B17" s="0" t="s">
         <x:v>69</x:v>
       </x:c>
-      <x:c r="C16" s="0" t="s">
+      <x:c r="C17" s="0" t="s">
         <x:v>70</x:v>
-      </x:c>
-      <x:c r="E16" s="0" t="s">
-        <x:v>71</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="17" spans="1:7">
-      <x:c r="B17" s="0" t="s">
-        <x:v>72</x:v>
       </x:c>
     </x:row>
     <x:row r="18" spans="1:7">
       <x:c r="B18" s="0" t="s">
-        <x:v>73</x:v>
-      </x:c>
-      <x:c r="C18" s="0" t="s">
-        <x:v>74</x:v>
-      </x:c>
-      <x:c r="E18" s="0" t="s">
-        <x:v>75</x:v>
+        <x:v>71</x:v>
       </x:c>
     </x:row>
     <x:row r="19" spans="1:7">
       <x:c r="B19" s="0" t="s">
-        <x:v>76</x:v>
+        <x:v>72</x:v>
       </x:c>
     </x:row>
     <x:row r="20" spans="1:7">
+      <x:c r="A20" s="0" t="s">
+        <x:v>73</x:v>
+      </x:c>
       <x:c r="B20" s="0" t="s">
-        <x:v>77</x:v>
+        <x:v>74</x:v>
       </x:c>
       <x:c r="C20" s="0" t="s">
-        <x:v>78</x:v>
-      </x:c>
-      <x:c r="E20" s="0" t="s">
-        <x:v>79</x:v>
+        <x:v>75</x:v>
       </x:c>
     </x:row>
     <x:row r="21" spans="1:7">
       <x:c r="B21" s="0" t="s">
-        <x:v>60</x:v>
+        <x:v>61</x:v>
       </x:c>
     </x:row>
     <x:row r="22" spans="1:7">
       <x:c r="B22" s="0" t="s">
-        <x:v>80</x:v>
-      </x:c>
-      <x:c r="C22" s="0" t="s">
-        <x:v>81</x:v>
-      </x:c>
-      <x:c r="E22" s="0" t="s">
-        <x:v>82</x:v>
+        <x:v>62</x:v>
       </x:c>
     </x:row>
     <x:row r="23" spans="1:7">
+      <x:c r="A23" s="0" t="s">
+        <x:v>76</x:v>
+      </x:c>
       <x:c r="B23" s="0" t="s">
-        <x:v>83</x:v>
+        <x:v>77</x:v>
+      </x:c>
+      <x:c r="C23" s="0" t="s">
+        <x:v>78</x:v>
       </x:c>
     </x:row>
     <x:row r="24" spans="1:7">
       <x:c r="B24" s="0" t="s">
-        <x:v>84</x:v>
-      </x:c>
-      <x:c r="C24" s="0" t="s">
-        <x:v>85</x:v>
-      </x:c>
-      <x:c r="E24" s="0" t="s">
-        <x:v>86</x:v>
+        <x:v>79</x:v>
       </x:c>
     </x:row>
     <x:row r="25" spans="1:7">
       <x:c r="B25" s="0" t="s">
-        <x:v>49</x:v>
+        <x:v>72</x:v>
       </x:c>
     </x:row>
     <x:row r="26" spans="1:7">
+      <x:c r="A26" s="0" t="s">
+        <x:v>80</x:v>
+      </x:c>
       <x:c r="B26" s="0" t="s">
-        <x:v>87</x:v>
+        <x:v>81</x:v>
       </x:c>
       <x:c r="C26" s="0" t="s">
-        <x:v>88</x:v>
-      </x:c>
-      <x:c r="E26" s="0" t="s">
-        <x:v>89</x:v>
+        <x:v>82</x:v>
       </x:c>
     </x:row>
     <x:row r="27" spans="1:7">
       <x:c r="B27" s="0" t="s">
-        <x:v>87</x:v>
-      </x:c>
-      <x:c r="C27" s="0" t="s">
-        <x:v>88</x:v>
-      </x:c>
-      <x:c r="E27" s="0" t="s">
-        <x:v>89</x:v>
+        <x:v>79</x:v>
       </x:c>
     </x:row>
     <x:row r="28" spans="1:7">
       <x:c r="B28" s="0" t="s">
-        <x:v>90</x:v>
+        <x:v>72</x:v>
       </x:c>
     </x:row>
     <x:row r="29" spans="1:7">
+      <x:c r="A29" s="0" t="s">
+        <x:v>83</x:v>
+      </x:c>
       <x:c r="B29" s="0" t="s">
-        <x:v>91</x:v>
+        <x:v>84</x:v>
       </x:c>
       <x:c r="C29" s="0" t="s">
-        <x:v>92</x:v>
-      </x:c>
-      <x:c r="E29" s="0" t="s">
-        <x:v>93</x:v>
+        <x:v>85</x:v>
       </x:c>
     </x:row>
     <x:row r="30" spans="1:7">
       <x:c r="B30" s="0" t="s">
-        <x:v>94</x:v>
+        <x:v>86</x:v>
       </x:c>
     </x:row>
     <x:row r="31" spans="1:7">
       <x:c r="B31" s="0" t="s">
-        <x:v>95</x:v>
+        <x:v>87</x:v>
       </x:c>
     </x:row>
     <x:row r="32" spans="1:7">
+      <x:c r="A32" s="0" t="s">
+        <x:v>88</x:v>
+      </x:c>
       <x:c r="B32" s="0" t="s">
-        <x:v>96</x:v>
+        <x:v>89</x:v>
       </x:c>
       <x:c r="C32" s="0" t="s">
-        <x:v>97</x:v>
-      </x:c>
-      <x:c r="E32" s="0" t="s">
-        <x:v>98</x:v>
+        <x:v>90</x:v>
       </x:c>
     </x:row>
     <x:row r="33" spans="1:7">
       <x:c r="B33" s="0" t="s">
-        <x:v>99</x:v>
+        <x:v>66</x:v>
       </x:c>
     </x:row>
     <x:row r="34" spans="1:7">
       <x:c r="B34" s="0" t="s">
-        <x:v>100</x:v>
+        <x:v>67</x:v>
       </x:c>
     </x:row>
     <x:row r="35" spans="1:7">
+      <x:c r="A35" s="0" t="s">
+        <x:v>91</x:v>
+      </x:c>
       <x:c r="B35" s="0" t="s">
-        <x:v>101</x:v>
+        <x:v>92</x:v>
       </x:c>
       <x:c r="C35" s="0" t="s">
-        <x:v>102</x:v>
-      </x:c>
-      <x:c r="E35" s="0" t="s">
-        <x:v>103</x:v>
+        <x:v>93</x:v>
       </x:c>
     </x:row>
     <x:row r="36" spans="1:7">
       <x:c r="B36" s="0" t="s">
-        <x:v>104</x:v>
+        <x:v>79</x:v>
       </x:c>
     </x:row>
     <x:row r="37" spans="1:7">
       <x:c r="B37" s="0" t="s">
-        <x:v>90</x:v>
+        <x:v>72</x:v>
       </x:c>
     </x:row>
     <x:row r="38" spans="1:7">
+      <x:c r="A38" s="0" t="s">
+        <x:v>94</x:v>
+      </x:c>
       <x:c r="B38" s="0" t="s">
-        <x:v>105</x:v>
+        <x:v>95</x:v>
       </x:c>
       <x:c r="C38" s="0" t="s">
-        <x:v>106</x:v>
-      </x:c>
-      <x:c r="E38" s="0" t="s">
-        <x:v>107</x:v>
+        <x:v>96</x:v>
       </x:c>
     </x:row>
     <x:row r="39" spans="1:7">
       <x:c r="B39" s="0" t="s">
-        <x:v>104</x:v>
+        <x:v>79</x:v>
       </x:c>
     </x:row>
     <x:row r="40" spans="1:7">
       <x:c r="B40" s="0" t="s">
-        <x:v>90</x:v>
+        <x:v>72</x:v>
       </x:c>
     </x:row>
     <x:row r="41" spans="1:7">
+      <x:c r="A41" s="0" t="s">
+        <x:v>97</x:v>
+      </x:c>
       <x:c r="B41" s="0" t="s">
-        <x:v>108</x:v>
+        <x:v>98</x:v>
       </x:c>
       <x:c r="C41" s="0" t="s">
-        <x:v>109</x:v>
-      </x:c>
-      <x:c r="E41" s="0" t="s">
-        <x:v>110</x:v>
+        <x:v>99</x:v>
       </x:c>
     </x:row>
     <x:row r="42" spans="1:7">
       <x:c r="B42" s="0" t="s">
-        <x:v>94</x:v>
+        <x:v>86</x:v>
       </x:c>
     </x:row>
     <x:row r="43" spans="1:7">
       <x:c r="B43" s="0" t="s">
-        <x:v>90</x:v>
+        <x:v>72</x:v>
       </x:c>
     </x:row>
     <x:row r="44" spans="1:7">
+      <x:c r="A44" s="0" t="s">
+        <x:v>100</x:v>
+      </x:c>
       <x:c r="B44" s="0" t="s">
-        <x:v>111</x:v>
+        <x:v>101</x:v>
       </x:c>
       <x:c r="C44" s="0" t="s">
-        <x:v>112</x:v>
-      </x:c>
-      <x:c r="E44" s="0" t="s">
-        <x:v>113</x:v>
+        <x:v>102</x:v>
       </x:c>
     </x:row>
     <x:row r="45" spans="1:7">
       <x:c r="B45" s="0" t="s">
-        <x:v>114</x:v>
+        <x:v>61</x:v>
       </x:c>
     </x:row>
     <x:row r="46" spans="1:7">
       <x:c r="B46" s="0" t="s">
-        <x:v>100</x:v>
+        <x:v>67</x:v>
       </x:c>
     </x:row>
     <x:row r="47" spans="1:7">
+      <x:c r="A47" s="0" t="s">
+        <x:v>103</x:v>
+      </x:c>
       <x:c r="B47" s="0" t="s">
-        <x:v>115</x:v>
+        <x:v>104</x:v>
       </x:c>
       <x:c r="C47" s="0" t="s">
-        <x:v>116</x:v>
-      </x:c>
-      <x:c r="E47" s="0" t="s">
-        <x:v>117</x:v>
+        <x:v>105</x:v>
       </x:c>
     </x:row>
     <x:row r="48" spans="1:7">
       <x:c r="B48" s="0" t="s">
-        <x:v>104</x:v>
+        <x:v>106</x:v>
       </x:c>
     </x:row>
     <x:row r="49" spans="1:7">
+      <x:c r="A49" s="0" t="s">
+        <x:v>107</x:v>
+      </x:c>
       <x:c r="B49" s="0" t="s">
-        <x:v>100</x:v>
+        <x:v>108</x:v>
+      </x:c>
+      <x:c r="C49" s="0" t="s">
+        <x:v>109</x:v>
       </x:c>
     </x:row>
     <x:row r="50" spans="1:7">
       <x:c r="B50" s="0" t="s">
-        <x:v>61</x:v>
-      </x:c>
-      <x:c r="C50" s="0" t="s">
-        <x:v>62</x:v>
-      </x:c>
-      <x:c r="E50" s="0" t="s">
-        <x:v>63</x:v>
+        <x:v>110</x:v>
       </x:c>
     </x:row>
     <x:row r="51" spans="1:7">
+      <x:c r="A51" s="0" t="s">
+        <x:v>111</x:v>
+      </x:c>
       <x:c r="B51" s="0" t="s">
-        <x:v>64</x:v>
+        <x:v>112</x:v>
+      </x:c>
+      <x:c r="C51" s="0" t="s">
+        <x:v>113</x:v>
       </x:c>
     </x:row>
     <x:row r="52" spans="1:7">
       <x:c r="B52" s="0" t="s">
-        <x:v>65</x:v>
-      </x:c>
-      <x:c r="C52" s="0" t="s">
-        <x:v>66</x:v>
-      </x:c>
-      <x:c r="E52" s="0" t="s">
-        <x:v>67</x:v>
+        <x:v>106</x:v>
       </x:c>
     </x:row>
     <x:row r="53" spans="1:7">
+      <x:c r="A53" s="0" t="s">
+        <x:v>114</x:v>
+      </x:c>
       <x:c r="B53" s="0" t="s">
-        <x:v>68</x:v>
+        <x:v>115</x:v>
+      </x:c>
+      <x:c r="C53" s="0" t="s">
+        <x:v>116</x:v>
       </x:c>
     </x:row>
     <x:row r="54" spans="1:7">
       <x:c r="B54" s="0" t="s">
-        <x:v>69</x:v>
-      </x:c>
-      <x:c r="C54" s="0" t="s">
-        <x:v>70</x:v>
-      </x:c>
-      <x:c r="E54" s="0" t="s">
-        <x:v>71</x:v>
+        <x:v>117</x:v>
       </x:c>
     </x:row>
     <x:row r="55" spans="1:7">
+      <x:c r="A55" s="0" t="s">
+        <x:v>118</x:v>
+      </x:c>
       <x:c r="B55" s="0" t="s">
-        <x:v>72</x:v>
+        <x:v>119</x:v>
+      </x:c>
+      <x:c r="C55" s="0" t="s">
+        <x:v>120</x:v>
       </x:c>
     </x:row>
     <x:row r="56" spans="1:7">
       <x:c r="B56" s="0" t="s">
-        <x:v>73</x:v>
-      </x:c>
-      <x:c r="C56" s="0" t="s">
-        <x:v>74</x:v>
-      </x:c>
-      <x:c r="E56" s="0" t="s">
-        <x:v>75</x:v>
+        <x:v>121</x:v>
       </x:c>
     </x:row>
     <x:row r="57" spans="1:7">
+      <x:c r="A57" s="0" t="s">
+        <x:v>122</x:v>
+      </x:c>
       <x:c r="B57" s="0" t="s">
-        <x:v>76</x:v>
+        <x:v>123</x:v>
+      </x:c>
+      <x:c r="C57" s="0" t="s">
+        <x:v>124</x:v>
       </x:c>
     </x:row>
     <x:row r="58" spans="1:7">
       <x:c r="B58" s="0" t="s">
-        <x:v>77</x:v>
-      </x:c>
-      <x:c r="C58" s="0" t="s">
-        <x:v>78</x:v>
-      </x:c>
-      <x:c r="E58" s="0" t="s">
-        <x:v>79</x:v>
+        <x:v>60</x:v>
       </x:c>
     </x:row>
     <x:row r="59" spans="1:7">
+      <x:c r="A59" s="0" t="s">
+        <x:v>125</x:v>
+      </x:c>
       <x:c r="B59" s="0" t="s">
-        <x:v>60</x:v>
+        <x:v>126</x:v>
+      </x:c>
+      <x:c r="C59" s="0" t="s">
+        <x:v>127</x:v>
       </x:c>
     </x:row>
     <x:row r="60" spans="1:7">
       <x:c r="B60" s="0" t="s">
-        <x:v>80</x:v>
-      </x:c>
-      <x:c r="C60" s="0" t="s">
-        <x:v>81</x:v>
-      </x:c>
-      <x:c r="E60" s="0" t="s">
-        <x:v>82</x:v>
+        <x:v>128</x:v>
       </x:c>
     </x:row>
     <x:row r="61" spans="1:7">
+      <x:c r="A61" s="0" t="s">
+        <x:v>129</x:v>
+      </x:c>
       <x:c r="B61" s="0" t="s">
-        <x:v>83</x:v>
+        <x:v>130</x:v>
+      </x:c>
+      <x:c r="C61" s="0" t="s">
+        <x:v>131</x:v>
       </x:c>
     </x:row>
     <x:row r="62" spans="1:7">
       <x:c r="B62" s="0" t="s">
-        <x:v>84</x:v>
-      </x:c>
-      <x:c r="C62" s="0" t="s">
-        <x:v>85</x:v>
-      </x:c>
-      <x:c r="E62" s="0" t="s">
-        <x:v>86</x:v>
+        <x:v>49</x:v>
       </x:c>
     </x:row>
     <x:row r="63" spans="1:7">
+      <x:c r="A63" s="0" t="s">
+        <x:v>132</x:v>
+      </x:c>
       <x:c r="B63" s="0" t="s">
-        <x:v>49</x:v>
+        <x:v>133</x:v>
+      </x:c>
+      <x:c r="C63" s="0" t="s">
+        <x:v>134</x:v>
       </x:c>
     </x:row>
     <x:row r="64" spans="1:7">
       <x:c r="B64" s="0" t="s">
-        <x:v>87</x:v>
+        <x:v>133</x:v>
       </x:c>
       <x:c r="C64" s="0" t="s">
-        <x:v>88</x:v>
+        <x:v>134</x:v>
       </x:c>
       <x:c r="E64" s="0" t="s">
-        <x:v>89</x:v>
+        <x:v>132</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1532,13 +1559,13 @@
       </x:c>
     </x:row>
     <x:row r="2" spans="1:7">
+      <x:c r="A2" s="0" t="s">
+        <x:v>42</x:v>
+      </x:c>
       <x:c r="B2" s="0" t="s">
-        <x:v>42</x:v>
+        <x:v>43</x:v>
       </x:c>
       <x:c r="C2" s="0" t="s">
-        <x:v>43</x:v>
-      </x:c>
-      <x:c r="E2" s="0" t="s">
         <x:v>44</x:v>
       </x:c>
     </x:row>
@@ -1548,13 +1575,13 @@
       </x:c>
     </x:row>
     <x:row r="4" spans="1:7">
+      <x:c r="A4" s="0" t="s">
+        <x:v>46</x:v>
+      </x:c>
       <x:c r="B4" s="0" t="s">
-        <x:v>46</x:v>
+        <x:v>47</x:v>
       </x:c>
       <x:c r="C4" s="0" t="s">
-        <x:v>47</x:v>
-      </x:c>
-      <x:c r="E4" s="0" t="s">
         <x:v>48</x:v>
       </x:c>
     </x:row>
@@ -1564,13 +1591,13 @@
       </x:c>
     </x:row>
     <x:row r="6" spans="1:7">
+      <x:c r="A6" s="0" t="s">
+        <x:v>50</x:v>
+      </x:c>
       <x:c r="B6" s="0" t="s">
-        <x:v>50</x:v>
+        <x:v>51</x:v>
       </x:c>
       <x:c r="C6" s="0" t="s">
-        <x:v>51</x:v>
-      </x:c>
-      <x:c r="E6" s="0" t="s">
         <x:v>52</x:v>
       </x:c>
     </x:row>
@@ -1580,13 +1607,13 @@
       </x:c>
     </x:row>
     <x:row r="8" spans="1:7">
+      <x:c r="A8" s="0" t="s">
+        <x:v>54</x:v>
+      </x:c>
       <x:c r="B8" s="0" t="s">
-        <x:v>54</x:v>
+        <x:v>55</x:v>
       </x:c>
       <x:c r="C8" s="0" t="s">
-        <x:v>55</x:v>
-      </x:c>
-      <x:c r="E8" s="0" t="s">
         <x:v>56</x:v>
       </x:c>
     </x:row>
@@ -1596,13 +1623,13 @@
       </x:c>
     </x:row>
     <x:row r="10" spans="1:7">
+      <x:c r="A10" s="0" t="s">
+        <x:v>57</x:v>
+      </x:c>
       <x:c r="B10" s="0" t="s">
-        <x:v>57</x:v>
+        <x:v>58</x:v>
       </x:c>
       <x:c r="C10" s="0" t="s">
-        <x:v>58</x:v>
-      </x:c>
-      <x:c r="E10" s="0" t="s">
         <x:v>59</x:v>
       </x:c>
     </x:row>
@@ -1615,409 +1642,391 @@
       <x:c r="B12" s="0" t="s">
         <x:v>61</x:v>
       </x:c>
-      <x:c r="C12" s="0" t="s">
-        <x:v>62</x:v>
-      </x:c>
-      <x:c r="E12" s="0" t="s">
-        <x:v>63</x:v>
-      </x:c>
     </x:row>
     <x:row r="13" spans="1:7">
       <x:c r="B13" s="0" t="s">
+        <x:v>62</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" spans="1:7">
+      <x:c r="A14" s="0" t="s">
+        <x:v>63</x:v>
+      </x:c>
+      <x:c r="B14" s="0" t="s">
         <x:v>64</x:v>
       </x:c>
-    </x:row>
-    <x:row r="14" spans="1:7">
-      <x:c r="B14" s="0" t="s">
+      <x:c r="C14" s="0" t="s">
         <x:v>65</x:v>
-      </x:c>
-      <x:c r="C14" s="0" t="s">
-        <x:v>66</x:v>
-      </x:c>
-      <x:c r="E14" s="0" t="s">
-        <x:v>67</x:v>
       </x:c>
     </x:row>
     <x:row r="15" spans="1:7">
       <x:c r="B15" s="0" t="s">
-        <x:v>68</x:v>
+        <x:v>66</x:v>
       </x:c>
     </x:row>
     <x:row r="16" spans="1:7">
       <x:c r="B16" s="0" t="s">
+        <x:v>67</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" spans="1:7">
+      <x:c r="A17" s="0" t="s">
+        <x:v>68</x:v>
+      </x:c>
+      <x:c r="B17" s="0" t="s">
         <x:v>69</x:v>
       </x:c>
-      <x:c r="C16" s="0" t="s">
+      <x:c r="C17" s="0" t="s">
         <x:v>70</x:v>
-      </x:c>
-      <x:c r="E16" s="0" t="s">
-        <x:v>71</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="17" spans="1:7">
-      <x:c r="B17" s="0" t="s">
-        <x:v>72</x:v>
       </x:c>
     </x:row>
     <x:row r="18" spans="1:7">
       <x:c r="B18" s="0" t="s">
-        <x:v>73</x:v>
-      </x:c>
-      <x:c r="C18" s="0" t="s">
-        <x:v>74</x:v>
-      </x:c>
-      <x:c r="E18" s="0" t="s">
-        <x:v>75</x:v>
+        <x:v>71</x:v>
       </x:c>
     </x:row>
     <x:row r="19" spans="1:7">
       <x:c r="B19" s="0" t="s">
-        <x:v>76</x:v>
+        <x:v>72</x:v>
       </x:c>
     </x:row>
     <x:row r="20" spans="1:7">
+      <x:c r="A20" s="0" t="s">
+        <x:v>73</x:v>
+      </x:c>
       <x:c r="B20" s="0" t="s">
-        <x:v>77</x:v>
+        <x:v>74</x:v>
       </x:c>
       <x:c r="C20" s="0" t="s">
-        <x:v>78</x:v>
-      </x:c>
-      <x:c r="E20" s="0" t="s">
-        <x:v>79</x:v>
+        <x:v>75</x:v>
       </x:c>
     </x:row>
     <x:row r="21" spans="1:7">
       <x:c r="B21" s="0" t="s">
-        <x:v>60</x:v>
+        <x:v>61</x:v>
       </x:c>
     </x:row>
     <x:row r="22" spans="1:7">
       <x:c r="B22" s="0" t="s">
-        <x:v>80</x:v>
-      </x:c>
-      <x:c r="C22" s="0" t="s">
-        <x:v>81</x:v>
-      </x:c>
-      <x:c r="E22" s="0" t="s">
-        <x:v>82</x:v>
+        <x:v>62</x:v>
       </x:c>
     </x:row>
     <x:row r="23" spans="1:7">
+      <x:c r="A23" s="0" t="s">
+        <x:v>76</x:v>
+      </x:c>
       <x:c r="B23" s="0" t="s">
-        <x:v>83</x:v>
+        <x:v>77</x:v>
+      </x:c>
+      <x:c r="C23" s="0" t="s">
+        <x:v>78</x:v>
       </x:c>
     </x:row>
     <x:row r="24" spans="1:7">
       <x:c r="B24" s="0" t="s">
-        <x:v>84</x:v>
-      </x:c>
-      <x:c r="C24" s="0" t="s">
-        <x:v>85</x:v>
-      </x:c>
-      <x:c r="E24" s="0" t="s">
-        <x:v>86</x:v>
+        <x:v>79</x:v>
       </x:c>
     </x:row>
     <x:row r="25" spans="1:7">
       <x:c r="B25" s="0" t="s">
-        <x:v>49</x:v>
+        <x:v>72</x:v>
       </x:c>
     </x:row>
     <x:row r="26" spans="1:7">
+      <x:c r="A26" s="0" t="s">
+        <x:v>80</x:v>
+      </x:c>
       <x:c r="B26" s="0" t="s">
-        <x:v>87</x:v>
+        <x:v>81</x:v>
       </x:c>
       <x:c r="C26" s="0" t="s">
-        <x:v>88</x:v>
-      </x:c>
-      <x:c r="E26" s="0" t="s">
-        <x:v>89</x:v>
+        <x:v>82</x:v>
       </x:c>
     </x:row>
     <x:row r="27" spans="1:7">
       <x:c r="B27" s="0" t="s">
-        <x:v>87</x:v>
-      </x:c>
-      <x:c r="C27" s="0" t="s">
-        <x:v>88</x:v>
-      </x:c>
-      <x:c r="E27" s="0" t="s">
-        <x:v>89</x:v>
+        <x:v>79</x:v>
       </x:c>
     </x:row>
     <x:row r="28" spans="1:7">
       <x:c r="B28" s="0" t="s">
-        <x:v>90</x:v>
+        <x:v>72</x:v>
       </x:c>
     </x:row>
     <x:row r="29" spans="1:7">
+      <x:c r="A29" s="0" t="s">
+        <x:v>83</x:v>
+      </x:c>
       <x:c r="B29" s="0" t="s">
-        <x:v>91</x:v>
+        <x:v>84</x:v>
       </x:c>
       <x:c r="C29" s="0" t="s">
-        <x:v>92</x:v>
-      </x:c>
-      <x:c r="E29" s="0" t="s">
-        <x:v>93</x:v>
+        <x:v>85</x:v>
       </x:c>
     </x:row>
     <x:row r="30" spans="1:7">
       <x:c r="B30" s="0" t="s">
-        <x:v>94</x:v>
+        <x:v>86</x:v>
       </x:c>
     </x:row>
     <x:row r="31" spans="1:7">
       <x:c r="B31" s="0" t="s">
-        <x:v>95</x:v>
+        <x:v>87</x:v>
       </x:c>
     </x:row>
     <x:row r="32" spans="1:7">
+      <x:c r="A32" s="0" t="s">
+        <x:v>88</x:v>
+      </x:c>
       <x:c r="B32" s="0" t="s">
-        <x:v>96</x:v>
+        <x:v>89</x:v>
       </x:c>
       <x:c r="C32" s="0" t="s">
-        <x:v>97</x:v>
-      </x:c>
-      <x:c r="E32" s="0" t="s">
-        <x:v>98</x:v>
+        <x:v>90</x:v>
       </x:c>
     </x:row>
     <x:row r="33" spans="1:7">
       <x:c r="B33" s="0" t="s">
-        <x:v>99</x:v>
+        <x:v>66</x:v>
       </x:c>
     </x:row>
     <x:row r="34" spans="1:7">
       <x:c r="B34" s="0" t="s">
-        <x:v>100</x:v>
+        <x:v>67</x:v>
       </x:c>
     </x:row>
     <x:row r="35" spans="1:7">
+      <x:c r="A35" s="0" t="s">
+        <x:v>91</x:v>
+      </x:c>
       <x:c r="B35" s="0" t="s">
-        <x:v>101</x:v>
+        <x:v>92</x:v>
       </x:c>
       <x:c r="C35" s="0" t="s">
-        <x:v>102</x:v>
-      </x:c>
-      <x:c r="E35" s="0" t="s">
-        <x:v>103</x:v>
+        <x:v>93</x:v>
       </x:c>
     </x:row>
     <x:row r="36" spans="1:7">
       <x:c r="B36" s="0" t="s">
-        <x:v>104</x:v>
+        <x:v>79</x:v>
       </x:c>
     </x:row>
     <x:row r="37" spans="1:7">
       <x:c r="B37" s="0" t="s">
-        <x:v>90</x:v>
+        <x:v>72</x:v>
       </x:c>
     </x:row>
     <x:row r="38" spans="1:7">
+      <x:c r="A38" s="0" t="s">
+        <x:v>94</x:v>
+      </x:c>
       <x:c r="B38" s="0" t="s">
-        <x:v>105</x:v>
+        <x:v>95</x:v>
       </x:c>
       <x:c r="C38" s="0" t="s">
-        <x:v>106</x:v>
-      </x:c>
-      <x:c r="E38" s="0" t="s">
-        <x:v>107</x:v>
+        <x:v>96</x:v>
       </x:c>
     </x:row>
     <x:row r="39" spans="1:7">
       <x:c r="B39" s="0" t="s">
-        <x:v>104</x:v>
+        <x:v>79</x:v>
       </x:c>
     </x:row>
     <x:row r="40" spans="1:7">
       <x:c r="B40" s="0" t="s">
-        <x:v>90</x:v>
+        <x:v>72</x:v>
       </x:c>
     </x:row>
     <x:row r="41" spans="1:7">
+      <x:c r="A41" s="0" t="s">
+        <x:v>97</x:v>
+      </x:c>
       <x:c r="B41" s="0" t="s">
-        <x:v>108</x:v>
+        <x:v>98</x:v>
       </x:c>
       <x:c r="C41" s="0" t="s">
-        <x:v>109</x:v>
-      </x:c>
-      <x:c r="E41" s="0" t="s">
-        <x:v>110</x:v>
+        <x:v>99</x:v>
       </x:c>
     </x:row>
     <x:row r="42" spans="1:7">
       <x:c r="B42" s="0" t="s">
-        <x:v>94</x:v>
+        <x:v>86</x:v>
       </x:c>
     </x:row>
     <x:row r="43" spans="1:7">
       <x:c r="B43" s="0" t="s">
-        <x:v>90</x:v>
+        <x:v>72</x:v>
       </x:c>
     </x:row>
     <x:row r="44" spans="1:7">
+      <x:c r="A44" s="0" t="s">
+        <x:v>100</x:v>
+      </x:c>
       <x:c r="B44" s="0" t="s">
-        <x:v>111</x:v>
+        <x:v>101</x:v>
       </x:c>
       <x:c r="C44" s="0" t="s">
-        <x:v>112</x:v>
-      </x:c>
-      <x:c r="E44" s="0" t="s">
-        <x:v>113</x:v>
+        <x:v>102</x:v>
       </x:c>
     </x:row>
     <x:row r="45" spans="1:7">
       <x:c r="B45" s="0" t="s">
-        <x:v>114</x:v>
+        <x:v>61</x:v>
       </x:c>
     </x:row>
     <x:row r="46" spans="1:7">
       <x:c r="B46" s="0" t="s">
-        <x:v>100</x:v>
+        <x:v>67</x:v>
       </x:c>
     </x:row>
     <x:row r="47" spans="1:7">
+      <x:c r="A47" s="0" t="s">
+        <x:v>103</x:v>
+      </x:c>
       <x:c r="B47" s="0" t="s">
-        <x:v>115</x:v>
+        <x:v>104</x:v>
       </x:c>
       <x:c r="C47" s="0" t="s">
-        <x:v>116</x:v>
-      </x:c>
-      <x:c r="E47" s="0" t="s">
-        <x:v>117</x:v>
+        <x:v>105</x:v>
       </x:c>
     </x:row>
     <x:row r="48" spans="1:7">
       <x:c r="B48" s="0" t="s">
-        <x:v>104</x:v>
+        <x:v>106</x:v>
       </x:c>
     </x:row>
     <x:row r="49" spans="1:7">
+      <x:c r="A49" s="0" t="s">
+        <x:v>107</x:v>
+      </x:c>
       <x:c r="B49" s="0" t="s">
-        <x:v>100</x:v>
+        <x:v>108</x:v>
+      </x:c>
+      <x:c r="C49" s="0" t="s">
+        <x:v>109</x:v>
       </x:c>
     </x:row>
     <x:row r="50" spans="1:7">
       <x:c r="B50" s="0" t="s">
-        <x:v>61</x:v>
-      </x:c>
-      <x:c r="C50" s="0" t="s">
-        <x:v>62</x:v>
-      </x:c>
-      <x:c r="E50" s="0" t="s">
-        <x:v>63</x:v>
+        <x:v>110</x:v>
       </x:c>
     </x:row>
     <x:row r="51" spans="1:7">
+      <x:c r="A51" s="0" t="s">
+        <x:v>111</x:v>
+      </x:c>
       <x:c r="B51" s="0" t="s">
-        <x:v>64</x:v>
+        <x:v>112</x:v>
+      </x:c>
+      <x:c r="C51" s="0" t="s">
+        <x:v>113</x:v>
       </x:c>
     </x:row>
     <x:row r="52" spans="1:7">
       <x:c r="B52" s="0" t="s">
-        <x:v>65</x:v>
-      </x:c>
-      <x:c r="C52" s="0" t="s">
-        <x:v>66</x:v>
-      </x:c>
-      <x:c r="E52" s="0" t="s">
-        <x:v>67</x:v>
+        <x:v>106</x:v>
       </x:c>
     </x:row>
     <x:row r="53" spans="1:7">
+      <x:c r="A53" s="0" t="s">
+        <x:v>114</x:v>
+      </x:c>
       <x:c r="B53" s="0" t="s">
-        <x:v>68</x:v>
+        <x:v>115</x:v>
+      </x:c>
+      <x:c r="C53" s="0" t="s">
+        <x:v>116</x:v>
       </x:c>
     </x:row>
     <x:row r="54" spans="1:7">
       <x:c r="B54" s="0" t="s">
-        <x:v>69</x:v>
-      </x:c>
-      <x:c r="C54" s="0" t="s">
-        <x:v>70</x:v>
-      </x:c>
-      <x:c r="E54" s="0" t="s">
-        <x:v>71</x:v>
+        <x:v>117</x:v>
       </x:c>
     </x:row>
     <x:row r="55" spans="1:7">
+      <x:c r="A55" s="0" t="s">
+        <x:v>118</x:v>
+      </x:c>
       <x:c r="B55" s="0" t="s">
-        <x:v>72</x:v>
+        <x:v>119</x:v>
+      </x:c>
+      <x:c r="C55" s="0" t="s">
+        <x:v>120</x:v>
       </x:c>
     </x:row>
     <x:row r="56" spans="1:7">
       <x:c r="B56" s="0" t="s">
-        <x:v>73</x:v>
-      </x:c>
-      <x:c r="C56" s="0" t="s">
-        <x:v>74</x:v>
-      </x:c>
-      <x:c r="E56" s="0" t="s">
-        <x:v>75</x:v>
+        <x:v>121</x:v>
       </x:c>
     </x:row>
     <x:row r="57" spans="1:7">
+      <x:c r="A57" s="0" t="s">
+        <x:v>122</x:v>
+      </x:c>
       <x:c r="B57" s="0" t="s">
-        <x:v>76</x:v>
+        <x:v>123</x:v>
+      </x:c>
+      <x:c r="C57" s="0" t="s">
+        <x:v>124</x:v>
       </x:c>
     </x:row>
     <x:row r="58" spans="1:7">
       <x:c r="B58" s="0" t="s">
-        <x:v>77</x:v>
-      </x:c>
-      <x:c r="C58" s="0" t="s">
-        <x:v>78</x:v>
-      </x:c>
-      <x:c r="E58" s="0" t="s">
-        <x:v>79</x:v>
+        <x:v>60</x:v>
       </x:c>
     </x:row>
     <x:row r="59" spans="1:7">
+      <x:c r="A59" s="0" t="s">
+        <x:v>125</x:v>
+      </x:c>
       <x:c r="B59" s="0" t="s">
-        <x:v>60</x:v>
+        <x:v>126</x:v>
+      </x:c>
+      <x:c r="C59" s="0" t="s">
+        <x:v>127</x:v>
       </x:c>
     </x:row>
     <x:row r="60" spans="1:7">
       <x:c r="B60" s="0" t="s">
-        <x:v>80</x:v>
-      </x:c>
-      <x:c r="C60" s="0" t="s">
-        <x:v>81</x:v>
-      </x:c>
-      <x:c r="E60" s="0" t="s">
-        <x:v>82</x:v>
+        <x:v>128</x:v>
       </x:c>
     </x:row>
     <x:row r="61" spans="1:7">
+      <x:c r="A61" s="0" t="s">
+        <x:v>129</x:v>
+      </x:c>
       <x:c r="B61" s="0" t="s">
-        <x:v>83</x:v>
+        <x:v>130</x:v>
+      </x:c>
+      <x:c r="C61" s="0" t="s">
+        <x:v>131</x:v>
       </x:c>
     </x:row>
     <x:row r="62" spans="1:7">
       <x:c r="B62" s="0" t="s">
-        <x:v>84</x:v>
-      </x:c>
-      <x:c r="C62" s="0" t="s">
-        <x:v>85</x:v>
-      </x:c>
-      <x:c r="E62" s="0" t="s">
-        <x:v>86</x:v>
+        <x:v>49</x:v>
       </x:c>
     </x:row>
     <x:row r="63" spans="1:7">
+      <x:c r="A63" s="0" t="s">
+        <x:v>132</x:v>
+      </x:c>
       <x:c r="B63" s="0" t="s">
-        <x:v>49</x:v>
+        <x:v>133</x:v>
+      </x:c>
+      <x:c r="C63" s="0" t="s">
+        <x:v>134</x:v>
       </x:c>
     </x:row>
     <x:row r="64" spans="1:7">
       <x:c r="B64" s="0" t="s">
-        <x:v>87</x:v>
+        <x:v>133</x:v>
       </x:c>
       <x:c r="C64" s="0" t="s">
-        <x:v>88</x:v>
+        <x:v>134</x:v>
       </x:c>
       <x:c r="E64" s="0" t="s">
-        <x:v>89</x:v>
+        <x:v>132</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>